<commit_message>
fixed Postman. Edited excel because of fixes
</commit_message>
<xml_diff>
--- a/testing/verification.xlsx
+++ b/testing/verification.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\calvi\Documents\CSCC01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\calvi\Documents\CSCC01\L01_03\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="83">
   <si>
     <t>Function</t>
   </si>
@@ -266,6 +266,15 @@
   <si>
     <t xml:space="preserve">500 internal error
 </t>
+  </si>
+  <si>
+    <t>Redirected to assignmentlist. Requested edit field was changed</t>
+  </si>
+  <si>
+    <t>New question was added to list from getQuestions</t>
+  </si>
+  <si>
+    <t>Previously created question has a changed name, question, and answer when grabbed from getQuestions</t>
   </si>
 </sst>
 </file>
@@ -834,7 +843,7 @@
         <v>32</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -902,7 +911,7 @@
         <v>49</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -938,7 +947,7 @@
         <v>56</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>